<commit_message>
fix(excel)!: accept independent input arrays
Allow input fields in nonadjacent ranges and independent row or column
orientations. Preserve blank positions, reject unequal entry counts and
reuse unchanged inputs after transposition.

BREAKING CHANGE: market inputs, loan schedules, discount mappings and
pricer settings take separate field arrays. Replace combined ranges with
individual field references. Loan settings take QS.LOAN.SETTINGS handles.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/context_pricing_example.xlsx
+++ b/bindings/excel/examples/context_pricing_example.xlsx
@@ -33,7 +33,8 @@
     <definedName name="Context_Originations">'4 Results'!$F$7:$F$9</definedName>
     <definedName name="Context_Pricer">'3 Contracts'!$B$13</definedName>
     <definedName name="Context_PV">'4 Results'!$B$7</definedName>
-    <definedName name="Context_QuoteRows">'1 Inputs'!$A$18:$B$30</definedName>
+    <definedName name="Context_QuoteIds">'1 Inputs'!$A$18:$A$30</definedName>
+    <definedName name="Context_QuoteMid">'1 Inputs'!$D$17:$P$17</definedName>
     <definedName name="Context_Rate">'1 Inputs'!$B$11</definedName>
     <definedName name="Context_Risk">'4 Results'!$A$161</definedName>
     <definedName name="Context_Root">'2 Contexts'!$B$7</definedName>
@@ -240,7 +241,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Same quote levels, next business date.</t>
+          <t>Same independent quote arrays, next business date.</t>
         </r>
       </text>
     </comment>
@@ -439,7 +440,7 @@
     <t>Identifier</t>
   </si>
   <si>
-    <t>Mid</t>
+    <t>Mid levels: independent row array</t>
   </si>
   <si>
     <t>FixedRateDeposit_EUR_ESTR_1D</t>
@@ -505,13 +506,13 @@
     <t>Date, currency, base index and optional quote side.</t>
   </si>
   <si>
-    <t>Market quotes</t>
+    <t>Independent quote arrays</t>
   </si>
   <si>
     <t>Curve from matching quotes</t>
   </si>
   <si>
-    <t>Inputs is B12:B13. Both formulas use Root; neither references the previous addition. You may instead use ADD.CURVE(root,index,quote_table) in one cell.</t>
+    <t>Inputs is B12:B13. Both formulas use Root; neither references the previous addition. You may instead use ADD.CURVE(root,index,identifiers,mid) in one cell.</t>
   </si>
   <si>
     <t>Second dated root</t>
@@ -559,7 +560,7 @@
     <t>Capture next market</t>
   </si>
   <si>
-    <t>Same quote levels, next business date.</t>
+    <t>Same independent quote arrays, next business date.</t>
   </si>
   <si>
     <t>First snapshot</t>
@@ -1422,34 +1423,35 @@
     <tabColor rgb="FF337AB7"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="62.7109375" style="1" customWidth="1"/>
+    <col min="4" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.25" customHeight="1">
+    <row r="1" spans="1:16" ht="38.25" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1">
+    <row r="2" spans="1:16" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
     </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1">
+    <row r="3" spans="1:16" ht="24" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:3" ht="36" customHeight="1">
+    <row r="4" spans="1:16" ht="36" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>30</v>
       </c>
@@ -1457,7 +1459,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1">
+    <row r="6" spans="1:16" ht="36" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -1468,7 +1470,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="32.25" customHeight="1">
+    <row r="7" spans="1:16" ht="32.25" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>35</v>
       </c>
@@ -1479,7 +1481,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32.25" customHeight="1">
+    <row r="8" spans="1:16" ht="32.25" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
@@ -1490,7 +1492,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32.25" customHeight="1">
+    <row r="9" spans="1:16" ht="32.25" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
@@ -1501,7 +1503,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32.25" customHeight="1">
+    <row r="10" spans="1:16" ht="32.25" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>44</v>
       </c>
@@ -1512,7 +1514,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32.25" customHeight="1">
+    <row r="11" spans="1:16" ht="32.25" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>46</v>
       </c>
@@ -1523,7 +1525,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="32.25" customHeight="1">
+    <row r="12" spans="1:16" ht="32.25" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>48</v>
       </c>
@@ -1534,123 +1536,139 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="36" customHeight="1">
+    <row r="16" spans="1:16" ht="24" customHeight="1">
+      <c r="D16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+    </row>
+    <row r="17" spans="1:16" ht="36" customHeight="1">
       <c r="A17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="B17" s="5"/>
       <c r="C17" s="5"/>
-    </row>
-    <row r="18" spans="1:3" ht="24" customHeight="1">
+      <c r="D17" s="12">
+        <v>0.029</v>
+      </c>
+      <c r="E17" s="12">
+        <v>0.0288</v>
+      </c>
+      <c r="F17" s="12">
+        <v>0.028</v>
+      </c>
+      <c r="G17" s="12">
+        <v>0.0265</v>
+      </c>
+      <c r="H17" s="12">
+        <v>0.025</v>
+      </c>
+      <c r="I17" s="12">
+        <v>0.0245</v>
+      </c>
+      <c r="J17" s="12">
+        <v>0.0243</v>
+      </c>
+      <c r="K17" s="12">
+        <v>0.0242</v>
+      </c>
+      <c r="L17" s="12">
+        <v>0.0245</v>
+      </c>
+      <c r="M17" s="12">
+        <v>0.0252</v>
+      </c>
+      <c r="N17" s="12">
+        <v>0.0258</v>
+      </c>
+      <c r="O17" s="12">
+        <v>0.0255</v>
+      </c>
+      <c r="P17" s="12">
+        <v>0.024</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="24" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="12">
-        <v>0.029</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="19" spans="1:16" ht="24" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="12">
-        <v>0.0288</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="20" spans="1:16" ht="24" customHeight="1">
       <c r="A20" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="12">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="21" spans="1:16" ht="24" customHeight="1">
       <c r="A21" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="12">
-        <v>0.0265</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="22" spans="1:16" ht="24" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="12">
-        <v>0.025</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="23" spans="1:16" ht="24" customHeight="1">
       <c r="A23" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="12">
-        <v>0.0245</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="24" spans="1:16" ht="24" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="12">
-        <v>0.0243</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="25" spans="1:16" ht="24" customHeight="1">
       <c r="A25" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="12">
-        <v>0.0242</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="26" spans="1:16" ht="24" customHeight="1">
       <c r="A26" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B26" s="12">
-        <v>0.0245</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="27" spans="1:16" ht="24" customHeight="1">
       <c r="A27" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="12">
-        <v>0.0252</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="28" spans="1:16" ht="24" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="12">
-        <v>0.0258</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="29" spans="1:16" ht="24" customHeight="1">
       <c r="A29" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B29" s="12">
-        <v>0.0255</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="24" customHeight="1">
+    </row>
+    <row r="30" spans="1:16" ht="24" customHeight="1">
       <c r="A30" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B30" s="12">
-        <v>0.024</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C3"/>
+    <mergeCell ref="D16:P16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
@@ -1741,7 +1759,7 @@
         <v>73</v>
       </c>
       <c r="B12" s="10" cm="1" t="str">
-        <f t="array" ref="B12">_xll.QS.CONTEXT.ADD.QUOTES(Context_Root,Context_QuoteRows)</f>
+        <f t="array" ref="B12">_xll.QS.CONTEXT.ADD.QUOTES(Context_Root,Context_QuoteIds,Context_QuoteMid)</f>
         <v/>
       </c>
     </row>
@@ -1791,7 +1809,7 @@
         <v>78</v>
       </c>
       <c r="B24" s="10" cm="1" t="str">
-        <f t="array" ref="B24">_xll.QS.CONTEXT.ADD.CURVE(Context_NextRoot,"ESTR",Context_QuoteRows)</f>
+        <f t="array" ref="B24">_xll.QS.CONTEXT.ADD.CURVE(Context_NextRoot,"ESTR",Context_QuoteIds,Context_QuoteMid)</f>
         <v/>
       </c>
     </row>

</xml_diff>